<commit_message>
Update Assignment 1 test cases spreadsheet
Replace Assignment 1 - Test cases.xlsx with updated version containing revised test cases. This changeset also accidentally adds the Excel temporary/lock file (~$Assignment 1 - Test cases.xlsx); consider removing that file and adding an appropriate .gitignore entry to prevent committing editor temp files in future.
</commit_message>
<xml_diff>
--- a/Assignment 1 - Test cases.xlsx
+++ b/Assignment 1 - Test cases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SLIIT\3year1sem\ITPM\Test assign\test_automation\IT3040-Assignment1-Singlish-Transliteration-Testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAC897DB-921A-44D6-9CC5-E584CAAA63AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99CFF9A4-8C33-44A8-A4CA-A44006D5FEBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="722" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -67,9 +67,6 @@
     <t>Neg_0003</t>
   </si>
   <si>
-    <t>dnma gedarata ynna.</t>
-  </si>
-  <si>
     <t>දැන්ම ගෙදරට යන්න.</t>
   </si>
   <si>
@@ -79,18 +76,12 @@
     <t>M</t>
   </si>
   <si>
-    <t>meka copy krla group akata danna.</t>
-  </si>
-  <si>
     <t>මේක copy කරලා group එකට දාන්න.</t>
   </si>
   <si>
     <t>Neg_0005</t>
   </si>
   <si>
-    <t>suba udasanak yaluwa!</t>
-  </si>
-  <si>
     <t>සුබ උදෑසනක් යාලුවා!</t>
   </si>
   <si>
@@ -100,9 +91,6 @@
     <t>Neg_0006</t>
   </si>
   <si>
-    <t>suba udeyk hamotama!</t>
-  </si>
-  <si>
     <t>සුබ උදෑසනක් හැමෝටම!</t>
   </si>
   <si>
@@ -112,9 +100,6 @@
     <t>Neg_0007</t>
   </si>
   <si>
-    <t>puluwannam mata call ekak denna.</t>
-  </si>
-  <si>
     <t>පුළුවන්නම් මට call එකක් දෙන්න.</t>
   </si>
   <si>
@@ -124,36 +109,24 @@
     <t>Neg_0008</t>
   </si>
   <si>
-    <t>karunakarala report eka ada ewanna.</t>
-  </si>
-  <si>
     <t>කරුණාකරලා report එක අද එවන්න.</t>
   </si>
   <si>
     <t>Neg_0009</t>
   </si>
   <si>
-    <t>hari mama ennam.</t>
-  </si>
-  <si>
     <t>හරි මම එන්නම්.</t>
   </si>
   <si>
     <t>Neg_0010</t>
   </si>
   <si>
-    <t>ow eka hari.</t>
-  </si>
-  <si>
     <t>ඔව් ඒක හරි.</t>
   </si>
   <si>
     <t>Neg_0011</t>
   </si>
   <si>
-    <t>tikak tikak theruna.</t>
-  </si>
-  <si>
     <t>ටිකක් ටිකක් තේරුණා.</t>
   </si>
   <si>
@@ -163,36 +136,24 @@
     <t>Neg_0012</t>
   </si>
   <si>
-    <t>epa epa dan katha karanna epa.</t>
-  </si>
-  <si>
     <t>එපා එපා දැන් කතා කරන්න එපා.</t>
   </si>
   <si>
     <t>Neg_0013</t>
   </si>
   <si>
-    <t>ei mehema une?</t>
-  </si>
-  <si>
     <t>ඇයි මෙහෙම උනේ?</t>
   </si>
   <si>
     <t>Neg_0014</t>
   </si>
   <si>
-    <t>ane... mata aka amathaka una!</t>
-  </si>
-  <si>
     <t>අනේ... මට ඒක අමතක උනා!</t>
   </si>
   <si>
     <t>Neg_0015</t>
   </si>
   <si>
-    <t>mn oyta heta msg ekak dannm.</t>
-  </si>
-  <si>
     <t>මං ඔයාට හෙට msg එකක් දාන්නම්.</t>
   </si>
   <si>
@@ -202,90 +163,60 @@
     <t>Neg_0016</t>
   </si>
   <si>
-    <t>oyge gedra kauda inne?</t>
-  </si>
-  <si>
     <t>ඔයාගේ ගෙදර කවුද ඉන්නේ?</t>
   </si>
   <si>
     <t>Neg_0017</t>
   </si>
   <si>
-    <t>mama ada lunch eka gedarin genawa.</t>
-  </si>
-  <si>
     <t>මම අද lunch එක ගෙදරින් ගෙනාවා.</t>
   </si>
   <si>
     <t>Neg_0018</t>
   </si>
   <si>
-    <t>ape sir assignment eka check kala.</t>
-  </si>
-  <si>
     <t>අපේ sir assignment එක check කළා.</t>
   </si>
   <si>
     <t>Neg_0019</t>
   </si>
   <si>
-    <t>mama dan ready to go inne.</t>
-  </si>
-  <si>
     <t>මම දැන් ready to go ඉන්නේ.</t>
   </si>
   <si>
     <t>Neg_0020</t>
   </si>
   <si>
-    <t>oya please wait karanna mama enakan.</t>
-  </si>
-  <si>
     <t>ඔයා please wait කරන්න මම එනකන්.</t>
   </si>
   <si>
     <t>Neg_0021</t>
   </si>
   <si>
-    <t>mage email eka update karanna.</t>
-  </si>
-  <si>
     <t>මගේ email එක update කරන්න.</t>
   </si>
   <si>
     <t>Neg_0022</t>
   </si>
   <si>
-    <t>password eka reset karanna puluwanda?</t>
-  </si>
-  <si>
     <t>password එක reset කරන්න පුළුවන්ද?</t>
   </si>
   <si>
     <t>Neg_0023</t>
   </si>
   <si>
-    <t>Teams meeting aka heta thiyenawa.</t>
-  </si>
-  <si>
     <t>Teams meeting එක හෙට තියෙනවා.</t>
   </si>
   <si>
     <t>Neg_0024</t>
   </si>
   <si>
-    <t>Telegram group akata msg ekak danna.</t>
-  </si>
-  <si>
     <t>Telegram group එකට msg එකක් දාන්න.</t>
   </si>
   <si>
     <t>Neg_0025</t>
   </si>
   <si>
-    <t>CV eka PDF widihata upload karanna.</t>
-  </si>
-  <si>
     <t>CV එක PDF විදිහට upload කරන්න.</t>
   </si>
   <si>
@@ -295,54 +226,36 @@
     <t>Neg_0026</t>
   </si>
   <si>
-    <t>ID card eka scan karala ewanna.</t>
-  </si>
-  <si>
     <t>ID card එක scan කරලා එවන්න.</t>
   </si>
   <si>
     <t>Neg_0027</t>
   </si>
   <si>
-    <t>heta practical ekata enna.</t>
-  </si>
-  <si>
     <t>හෙට practical එකට එන්න.</t>
   </si>
   <si>
     <t>Neg_0028</t>
   </si>
   <si>
-    <t>lab report eka submit karada?</t>
-  </si>
-  <si>
     <t>lab report එක submit කරාද?</t>
   </si>
   <si>
     <t>Neg_0029</t>
   </si>
   <si>
-    <t>api heta Kandy walata yanawa.</t>
-  </si>
-  <si>
     <t>අපි හෙට Kandy වලට යනවා.</t>
   </si>
   <si>
     <t>Neg_0030</t>
   </si>
   <si>
-    <t>mama Colombo Fort eken bus ekata nagga.</t>
-  </si>
-  <si>
     <t>මම Colombo Fort එකෙන් bus එකට නැග්ගා.</t>
   </si>
   <si>
     <t>Neg_0031</t>
   </si>
   <si>
-    <t>Kasun ada exam ekata awe na.</t>
-  </si>
-  <si>
     <t>Kasun අද exam එකට ආවේ නෑ.</t>
   </si>
   <si>
@@ -352,9 +265,6 @@
     <t>Neg_0032</t>
   </si>
   <si>
-    <t>Nethmi presentation eka lassanata kala.</t>
-  </si>
-  <si>
     <t>Nethmi presentation එක ලස්සනට කළා.</t>
   </si>
   <si>
@@ -364,36 +274,24 @@
     <t>Neg_0033</t>
   </si>
   <si>
-    <t>mata 2nd attempt ekata register wenna one.</t>
-  </si>
-  <si>
     <t>මට 2nd attempt එකට register වෙන්න ඕනේ.</t>
   </si>
   <si>
     <t>Neg_0034</t>
   </si>
   <si>
-    <t>lamai 25k class akata awa.</t>
-  </si>
-  <si>
     <t>ළමයි 25ක් class එකට ආවා.</t>
   </si>
   <si>
     <t>Neg_0035</t>
   </si>
   <si>
-    <t>mata Rs. 1500k transfer karanna.</t>
-  </si>
-  <si>
     <t>මට Rs. 1500ක් transfer කරන්න.</t>
   </si>
   <si>
     <t>Neg_0036</t>
   </si>
   <si>
-    <t>dollar 20k gewanna una.</t>
-  </si>
-  <si>
     <t>dollar 20ක් ගෙවන්න උනා.</t>
   </si>
   <si>
@@ -403,18 +301,12 @@
     <t>Neg_0037</t>
   </si>
   <si>
-    <t>class eka 8.30pm patan gannawa.</t>
-  </si>
-  <si>
     <t>class එක 8.30pm පටන් ගන්නවා.</t>
   </si>
   <si>
     <t>Neg_0038</t>
   </si>
   <si>
-    <t>mata 10:15AM walata mathak karanna.</t>
-  </si>
-  <si>
     <t>මට 10:15AM වෙලාවට මතක් කරන්න.</t>
   </si>
   <si>
@@ -424,45 +316,30 @@
     <t>Neg_0039</t>
   </si>
   <si>
-    <t>exam eka 2026-05-12 wenida thiyenawa.</t>
-  </si>
-  <si>
     <t>exam එක 2026-05-12 වෙනිදා තියෙනවා.</t>
   </si>
   <si>
     <t>Neg_0040</t>
   </si>
   <si>
-    <t>assignment eka March 3ta kalin denna.</t>
-  </si>
-  <si>
     <t>assignment එක March 3ට කලින් දෙන්න.</t>
   </si>
   <si>
     <t>Neg_0041</t>
   </si>
   <si>
-    <t>mata 500g seeni genna.</t>
-  </si>
-  <si>
     <t>මට 500g සීනි ගේන්න.</t>
   </si>
   <si>
     <t>Neg_0042</t>
   </si>
   <si>
-    <t>bike eka 5km withara giya.</t>
-  </si>
-  <si>
     <t>bike එක 5km විතර ගියා.</t>
   </si>
   <si>
     <t>Neg_0043</t>
   </si>
   <si>
-    <t>patta machan oya wede goda dagaththa.</t>
-  </si>
-  <si>
     <t>පට්ට මචං ඔයා වැඩේ ගොඩ දාගත්තා.</t>
   </si>
   <si>
@@ -472,18 +349,12 @@
     <t>Neg_0044</t>
   </si>
   <si>
-    <t>ado mata podi help ekak one.</t>
-  </si>
-  <si>
     <t>අඩෝ මට පොඩි help එකක් ඕනේ.</t>
   </si>
   <si>
     <t>Neg_0045</t>
   </si>
   <si>
-    <t>me link eka open karanna: https://sliit.lk</t>
-  </si>
-  <si>
     <t>මේ link එක open කරන්න: https://sliit.lk</t>
   </si>
   <si>
@@ -493,9 +364,6 @@
     <t>Neg_0046</t>
   </si>
   <si>
-    <t>mata email ekak danna: raki2026@gmail.com</t>
-  </si>
-  <si>
     <t>මට email එකක් දාන්න: raki2026@gmail.com</t>
   </si>
   <si>
@@ -505,18 +373,12 @@
     <t>Neg_0047</t>
   </si>
   <si>
-    <t>mata dan hina yanawa 😂</t>
-  </si>
-  <si>
     <t>මට දැන් හිනා යනවා 😂</t>
   </si>
   <si>
     <t>Neg_0048</t>
   </si>
   <si>
-    <t>oya wede hodata kala ❤️</t>
-  </si>
-  <si>
     <t>ඔයා වැඩේ හොඳට කළා ❤️</t>
   </si>
   <si>
@@ -554,6 +416,144 @@
   </si>
   <si>
     <t>ada class ek tiyenwada?</t>
+  </si>
+  <si>
+    <t>dnm gedrta ynn.</t>
+  </si>
+  <si>
+    <t>mek copy krl group akt dnna.</t>
+  </si>
+  <si>
+    <t>sub udasanak yaluwa!</t>
+  </si>
+  <si>
+    <t>sub udeyk hamotama!</t>
+  </si>
+  <si>
+    <t>puluwnnam mt call ekk denna.</t>
+  </si>
+  <si>
+    <t>karunkarala report ek ada ewnna.</t>
+  </si>
+  <si>
+    <t>hri man ennam.</t>
+  </si>
+  <si>
+    <t>ow ek hari.</t>
+  </si>
+  <si>
+    <t>tikk tikk teruna.</t>
+  </si>
+  <si>
+    <t>ep ep dn kata karnna epa.</t>
+  </si>
+  <si>
+    <t>aye mehma une?</t>
+  </si>
+  <si>
+    <t>ane... mt ak amthka una!</t>
+  </si>
+  <si>
+    <t>mn oyt heta msg ekk dnnm.</t>
+  </si>
+  <si>
+    <t>oyge gedr kuda inne?</t>
+  </si>
+  <si>
+    <t>man ada lunch eka gedarin genawa.</t>
+  </si>
+  <si>
+    <t>ape sir assignment ek check kl.</t>
+  </si>
+  <si>
+    <t>man dn ready to go inne.</t>
+  </si>
+  <si>
+    <t>oya please wait karann mma enkn.</t>
+  </si>
+  <si>
+    <t>mge email ek update karnn.</t>
+  </si>
+  <si>
+    <t>password ek reset krnna puluwanda?</t>
+  </si>
+  <si>
+    <t>Teams meeting ak heta thiyenawa.</t>
+  </si>
+  <si>
+    <t>Telegram group akt msg ekk danna.</t>
+  </si>
+  <si>
+    <t>CV ek PDF widihta upload karnna.</t>
+  </si>
+  <si>
+    <t>ID card ek scan karla ewnna.</t>
+  </si>
+  <si>
+    <t>het practical ekta enna.</t>
+  </si>
+  <si>
+    <t>lab report ek submit karda?</t>
+  </si>
+  <si>
+    <t>api heta Kandy wlt ynawa.</t>
+  </si>
+  <si>
+    <t>mn Colombo Fort eken bus ekata nagga.</t>
+  </si>
+  <si>
+    <t>Kasun ada exam ekt awe na.</t>
+  </si>
+  <si>
+    <t>Nethmi presentation ek lssnt kala.</t>
+  </si>
+  <si>
+    <t>mt 2nd attempt ekt register wenna one.</t>
+  </si>
+  <si>
+    <t>lamai 25k class ekt awa.</t>
+  </si>
+  <si>
+    <t>mt Rs. 1500k transfer krnna.</t>
+  </si>
+  <si>
+    <t>Dollar 20k gewnna una.</t>
+  </si>
+  <si>
+    <t>class ek 8.30pm ptn gnnawa.</t>
+  </si>
+  <si>
+    <t>mt 10:15AM wlt mtk krnna.</t>
+  </si>
+  <si>
+    <t>exam ek 2026-05-12 wenida thiyenwa.</t>
+  </si>
+  <si>
+    <t>assignment ek March 3t klin denna.</t>
+  </si>
+  <si>
+    <t>mt 500g sini genna.</t>
+  </si>
+  <si>
+    <t>bike ek 5km witra giya.</t>
+  </si>
+  <si>
+    <t>ptt machan oya wede goda dgththa.</t>
+  </si>
+  <si>
+    <t>ado mt podi help ekk one.</t>
+  </si>
+  <si>
+    <t>me link ek open krnna: https://sliit.lk</t>
+  </si>
+  <si>
+    <t>mt email ekk danna: raki2026@gmail.com</t>
+  </si>
+  <si>
+    <t>mt dn hina ynwa 😂</t>
+  </si>
+  <si>
+    <t>oya wede hodt kala ❤️</t>
   </si>
 </sst>
 </file>
@@ -700,13 +700,13 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
@@ -1032,7 +1032,7 @@
         <v>7</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>176</v>
+        <v>130</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>8</v>
@@ -1040,7 +1040,7 @@
       <c r="E2" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="F2" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1076,15 +1076,15 @@
         <v>7</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>177</v>
+        <v>131</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="E6" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="F6" s="8" t="s">
+      <c r="F6" s="5" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1120,15 +1120,15 @@
         <v>7</v>
       </c>
       <c r="C10" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="D10" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D10" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="F10" s="8" t="s">
+      <c r="E10" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="F10" s="5" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1158,21 +1158,21 @@
     </row>
     <row r="14" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="C14" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="D14" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C14" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E14" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="F14" s="8" t="s">
+      <c r="E14" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="F14" s="5" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1202,21 +1202,21 @@
     </row>
     <row r="18" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>22</v>
+        <v>134</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E18" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="F18" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="E18" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="F18" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1246,21 +1246,21 @@
     </row>
     <row r="22" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>26</v>
+        <v>135</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E22" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="F22" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="E22" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="F22" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1290,21 +1290,21 @@
     </row>
     <row r="26" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>30</v>
+        <v>136</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="E26" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="F26" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="E26" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="F26" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1334,21 +1334,21 @@
     </row>
     <row r="30" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>34</v>
+        <v>137</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="E30" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="F30" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="E30" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="F30" s="5" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1378,21 +1378,21 @@
     </row>
     <row r="34" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="B34" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>37</v>
+        <v>138</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="E34" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="F34" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="E34" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="F34" s="5" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1422,21 +1422,21 @@
     </row>
     <row r="38" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="B38" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>40</v>
+        <v>139</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="E38" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="F38" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="E38" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="F38" s="5" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1466,21 +1466,21 @@
     </row>
     <row r="42" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="B42" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>43</v>
+        <v>140</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="E42" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="F42" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="E42" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="F42" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1510,21 +1510,21 @@
     </row>
     <row r="46" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="B46" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>47</v>
+        <v>141</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="E46" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="F46" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="E46" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="F46" s="5" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1554,21 +1554,21 @@
     </row>
     <row r="50" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="B50" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>50</v>
+        <v>142</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="E50" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="F50" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="E50" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="F50" s="5" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1598,21 +1598,21 @@
     </row>
     <row r="54" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="B54" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>53</v>
+        <v>143</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="E54" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="F54" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="E54" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="F54" s="5" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1642,21 +1642,21 @@
     </row>
     <row r="58" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" s="2" t="s">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="B58" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>56</v>
+        <v>144</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="E58" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="F58" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="E58" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="F58" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1686,21 +1686,21 @@
     </row>
     <row r="62" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A62" s="2" t="s">
-        <v>59</v>
+        <v>46</v>
       </c>
       <c r="B62" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>60</v>
+        <v>145</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="E62" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="F62" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="E62" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="F62" s="5" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1730,21 +1730,21 @@
     </row>
     <row r="66" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A66" s="2" t="s">
-        <v>62</v>
+        <v>48</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>63</v>
+        <v>146</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="E66" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="F66" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="E66" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="F66" s="5" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1774,21 +1774,21 @@
     </row>
     <row r="70" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A70" s="2" t="s">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>66</v>
+        <v>147</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="E70" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="F70" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="E70" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="F70" s="5" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1818,21 +1818,21 @@
     </row>
     <row r="74" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A74" s="2" t="s">
-        <v>68</v>
+        <v>52</v>
       </c>
       <c r="B74" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>69</v>
+        <v>148</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="E74" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="F74" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="E74" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="F74" s="5" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1862,21 +1862,21 @@
     </row>
     <row r="78" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A78" s="2" t="s">
-        <v>71</v>
+        <v>54</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>72</v>
+        <v>149</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="E78" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="F78" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="E78" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="F78" s="5" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1906,21 +1906,21 @@
     </row>
     <row r="82" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A82" s="2" t="s">
-        <v>74</v>
+        <v>56</v>
       </c>
       <c r="B82" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>75</v>
+        <v>150</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="E82" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="F82" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="E82" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="F82" s="5" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1950,21 +1950,21 @@
     </row>
     <row r="86" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A86" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C86" s="2" t="s">
-        <v>78</v>
+        <v>151</v>
       </c>
       <c r="D86" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="E86" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="F86" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="E86" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="F86" s="5" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1994,21 +1994,21 @@
     </row>
     <row r="90" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A90" s="2" t="s">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C90" s="2" t="s">
-        <v>81</v>
+        <v>152</v>
       </c>
       <c r="D90" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="E90" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="F90" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="E90" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="F90" s="5" t="s">
         <v>13</v>
       </c>
     </row>
@@ -2038,21 +2038,21 @@
     </row>
     <row r="94" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A94" s="2" t="s">
-        <v>83</v>
+        <v>62</v>
       </c>
       <c r="B94" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C94" s="2" t="s">
-        <v>84</v>
+        <v>153</v>
       </c>
       <c r="D94" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="E94" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="F94" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="E94" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="F94" s="5" t="s">
         <v>13</v>
       </c>
     </row>
@@ -2082,21 +2082,21 @@
     </row>
     <row r="98" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A98" s="2" t="s">
-        <v>86</v>
+        <v>64</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C98" s="2" t="s">
-        <v>87</v>
+        <v>154</v>
       </c>
       <c r="D98" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="E98" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="F98" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="E98" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="F98" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2126,21 +2126,21 @@
     </row>
     <row r="102" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A102" s="2" t="s">
-        <v>90</v>
+        <v>67</v>
       </c>
       <c r="B102" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C102" s="2" t="s">
-        <v>91</v>
+        <v>155</v>
       </c>
       <c r="D102" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="E102" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="F102" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="E102" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="F102" s="5" t="s">
         <v>13</v>
       </c>
     </row>
@@ -2170,21 +2170,21 @@
     </row>
     <row r="106" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A106" s="2" t="s">
-        <v>93</v>
+        <v>69</v>
       </c>
       <c r="B106" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C106" s="2" t="s">
-        <v>94</v>
+        <v>156</v>
       </c>
       <c r="D106" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="E106" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="F106" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="E106" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="F106" s="5" t="s">
         <v>13</v>
       </c>
     </row>
@@ -2214,21 +2214,21 @@
     </row>
     <row r="110" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A110" s="2" t="s">
-        <v>96</v>
+        <v>71</v>
       </c>
       <c r="B110" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C110" s="2" t="s">
-        <v>97</v>
+        <v>157</v>
       </c>
       <c r="D110" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="E110" s="5" t="s">
-        <v>98</v>
-      </c>
-      <c r="F110" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="E110" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="F110" s="5" t="s">
         <v>13</v>
       </c>
     </row>
@@ -2258,21 +2258,21 @@
     </row>
     <row r="114" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A114" s="2" t="s">
-        <v>99</v>
+        <v>73</v>
       </c>
       <c r="B114" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C114" s="2" t="s">
-        <v>100</v>
+        <v>158</v>
       </c>
       <c r="D114" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="E114" s="5" t="s">
-        <v>101</v>
-      </c>
-      <c r="F114" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="E114" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="F114" s="5" t="s">
         <v>13</v>
       </c>
     </row>
@@ -2302,21 +2302,21 @@
     </row>
     <row r="118" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A118" s="2" t="s">
-        <v>102</v>
+        <v>75</v>
       </c>
       <c r="B118" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C118" s="2" t="s">
-        <v>103</v>
+        <v>159</v>
       </c>
       <c r="D118" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="E118" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="F118" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="E118" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="F118" s="5" t="s">
         <v>13</v>
       </c>
     </row>
@@ -2346,21 +2346,21 @@
     </row>
     <row r="122" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A122" s="2" t="s">
-        <v>105</v>
+        <v>77</v>
       </c>
       <c r="B122" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C122" s="2" t="s">
-        <v>106</v>
+        <v>160</v>
       </c>
       <c r="D122" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="E122" s="5" t="s">
-        <v>108</v>
-      </c>
-      <c r="F122" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="E122" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="F122" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2390,21 +2390,21 @@
     </row>
     <row r="126" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A126" s="2" t="s">
-        <v>109</v>
+        <v>80</v>
       </c>
       <c r="B126" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C126" s="2" t="s">
-        <v>110</v>
+        <v>161</v>
       </c>
       <c r="D126" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="E126" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="F126" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="E126" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="F126" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2434,21 +2434,21 @@
     </row>
     <row r="130" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A130" s="2" t="s">
-        <v>113</v>
+        <v>83</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C130" s="2" t="s">
-        <v>114</v>
+        <v>162</v>
       </c>
       <c r="D130" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="E130" s="5" t="s">
-        <v>115</v>
-      </c>
-      <c r="F130" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="E130" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="F130" s="5" t="s">
         <v>13</v>
       </c>
     </row>
@@ -2478,21 +2478,21 @@
     </row>
     <row r="134" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A134" s="2" t="s">
-        <v>116</v>
+        <v>85</v>
       </c>
       <c r="B134" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C134" s="2" t="s">
-        <v>117</v>
+        <v>163</v>
       </c>
       <c r="D134" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="E134" s="5" t="s">
-        <v>118</v>
-      </c>
-      <c r="F134" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="E134" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="F134" s="5" t="s">
         <v>13</v>
       </c>
     </row>
@@ -2522,21 +2522,21 @@
     </row>
     <row r="138" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A138" s="2" t="s">
-        <v>119</v>
+        <v>87</v>
       </c>
       <c r="B138" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C138" s="2" t="s">
-        <v>120</v>
+        <v>164</v>
       </c>
       <c r="D138" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="E138" s="5" t="s">
-        <v>121</v>
-      </c>
-      <c r="F138" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="E138" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="F138" s="5" t="s">
         <v>13</v>
       </c>
     </row>
@@ -2566,21 +2566,21 @@
     </row>
     <row r="142" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A142" s="2" t="s">
-        <v>122</v>
+        <v>89</v>
       </c>
       <c r="B142" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C142" s="2" t="s">
-        <v>123</v>
+        <v>165</v>
       </c>
       <c r="D142" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="E142" s="5" t="s">
-        <v>125</v>
-      </c>
-      <c r="F142" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="E142" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="F142" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2610,21 +2610,21 @@
     </row>
     <row r="146" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A146" s="2" t="s">
-        <v>126</v>
+        <v>92</v>
       </c>
       <c r="B146" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C146" s="2" t="s">
-        <v>127</v>
+        <v>166</v>
       </c>
       <c r="D146" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="E146" s="5" t="s">
-        <v>128</v>
-      </c>
-      <c r="F146" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="E146" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="F146" s="5" t="s">
         <v>13</v>
       </c>
     </row>
@@ -2654,21 +2654,21 @@
     </row>
     <row r="150" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A150" s="2" t="s">
-        <v>129</v>
+        <v>94</v>
       </c>
       <c r="B150" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C150" s="2" t="s">
-        <v>130</v>
+        <v>167</v>
       </c>
       <c r="D150" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="E150" s="5" t="s">
-        <v>132</v>
-      </c>
-      <c r="F150" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="E150" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="F150" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2698,21 +2698,21 @@
     </row>
     <row r="154" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A154" s="2" t="s">
-        <v>133</v>
+        <v>97</v>
       </c>
       <c r="B154" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C154" s="2" t="s">
-        <v>134</v>
+        <v>168</v>
       </c>
       <c r="D154" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="E154" s="5" t="s">
-        <v>135</v>
-      </c>
-      <c r="F154" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="E154" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="F154" s="5" t="s">
         <v>13</v>
       </c>
     </row>
@@ -2742,21 +2742,21 @@
     </row>
     <row r="158" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A158" s="2" t="s">
-        <v>136</v>
+        <v>99</v>
       </c>
       <c r="B158" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C158" s="2" t="s">
-        <v>137</v>
+        <v>169</v>
       </c>
       <c r="D158" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="E158" s="5" t="s">
-        <v>138</v>
-      </c>
-      <c r="F158" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="E158" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="F158" s="5" t="s">
         <v>13</v>
       </c>
     </row>
@@ -2786,21 +2786,21 @@
     </row>
     <row r="162" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A162" s="2" t="s">
-        <v>139</v>
+        <v>101</v>
       </c>
       <c r="B162" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C162" s="2" t="s">
-        <v>140</v>
+        <v>170</v>
       </c>
       <c r="D162" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="E162" s="5" t="s">
-        <v>141</v>
-      </c>
-      <c r="F162" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="E162" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="F162" s="5" t="s">
         <v>13</v>
       </c>
     </row>
@@ -2830,21 +2830,21 @@
     </row>
     <row r="166" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A166" s="2" t="s">
-        <v>142</v>
+        <v>103</v>
       </c>
       <c r="B166" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C166" s="2" t="s">
-        <v>143</v>
+        <v>171</v>
       </c>
       <c r="D166" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="E166" s="5" t="s">
-        <v>144</v>
-      </c>
-      <c r="F166" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="E166" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="F166" s="5" t="s">
         <v>13</v>
       </c>
     </row>
@@ -2874,21 +2874,21 @@
     </row>
     <row r="170" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A170" s="2" t="s">
-        <v>145</v>
+        <v>105</v>
       </c>
       <c r="B170" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C170" s="2" t="s">
-        <v>146</v>
+        <v>172</v>
       </c>
       <c r="D170" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="E170" s="5" t="s">
-        <v>148</v>
-      </c>
-      <c r="F170" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="E170" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="F170" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2918,21 +2918,21 @@
     </row>
     <row r="174" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A174" s="2" t="s">
-        <v>149</v>
+        <v>108</v>
       </c>
       <c r="B174" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C174" s="2" t="s">
-        <v>150</v>
+        <v>173</v>
       </c>
       <c r="D174" s="2" t="s">
-        <v>151</v>
-      </c>
-      <c r="E174" s="5" t="s">
-        <v>151</v>
-      </c>
-      <c r="F174" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="E174" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="F174" s="5" t="s">
         <v>13</v>
       </c>
     </row>
@@ -2962,21 +2962,21 @@
     </row>
     <row r="178" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A178" s="2" t="s">
-        <v>152</v>
+        <v>110</v>
       </c>
       <c r="B178" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C178" s="2" t="s">
-        <v>153</v>
+        <v>174</v>
       </c>
       <c r="D178" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="E178" s="5" t="s">
-        <v>155</v>
-      </c>
-      <c r="F178" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="E178" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="F178" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -3006,21 +3006,21 @@
     </row>
     <row r="182" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A182" s="2" t="s">
-        <v>156</v>
+        <v>113</v>
       </c>
       <c r="B182" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C182" s="2" t="s">
-        <v>157</v>
+        <v>175</v>
       </c>
       <c r="D182" s="2" t="s">
-        <v>158</v>
-      </c>
-      <c r="E182" s="5" t="s">
-        <v>159</v>
-      </c>
-      <c r="F182" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="E182" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="F182" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -3050,21 +3050,21 @@
     </row>
     <row r="186" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A186" s="2" t="s">
-        <v>160</v>
+        <v>116</v>
       </c>
       <c r="B186" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C186" s="2" t="s">
-        <v>161</v>
+        <v>176</v>
       </c>
       <c r="D186" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="E186" s="5" t="s">
-        <v>162</v>
-      </c>
-      <c r="F186" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="E186" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="F186" s="5" t="s">
         <v>13</v>
       </c>
     </row>
@@ -3094,21 +3094,21 @@
     </row>
     <row r="190" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A190" s="2" t="s">
-        <v>163</v>
+        <v>118</v>
       </c>
       <c r="B190" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C190" s="2" t="s">
-        <v>164</v>
+        <v>177</v>
       </c>
       <c r="D190" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="E190" s="5" t="s">
-        <v>166</v>
-      </c>
-      <c r="F190" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="E190" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="F190" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -3138,21 +3138,21 @@
     </row>
     <row r="194" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A194" s="2" t="s">
-        <v>167</v>
+        <v>121</v>
       </c>
       <c r="B194" s="2" t="s">
-        <v>168</v>
+        <v>122</v>
       </c>
       <c r="C194" s="2" t="s">
-        <v>169</v>
+        <v>123</v>
       </c>
       <c r="D194" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="E194" s="5" t="s">
-        <v>171</v>
-      </c>
-      <c r="F194" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="E194" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="F194" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -3182,21 +3182,21 @@
     </row>
     <row r="198" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A198" s="2" t="s">
-        <v>172</v>
+        <v>126</v>
       </c>
       <c r="B198" s="2" t="s">
-        <v>168</v>
+        <v>122</v>
       </c>
       <c r="C198" s="2" t="s">
-        <v>173</v>
+        <v>127</v>
       </c>
       <c r="D198" s="2" t="s">
-        <v>174</v>
-      </c>
-      <c r="E198" s="5" t="s">
-        <v>175</v>
-      </c>
-      <c r="F198" s="8" t="s">
+        <v>128</v>
+      </c>
+      <c r="E198" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="F198" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -3226,6 +3226,282 @@
     </row>
   </sheetData>
   <mergeCells count="300">
+    <mergeCell ref="A118:A121"/>
+    <mergeCell ref="C14:C17"/>
+    <mergeCell ref="B66:B69"/>
+    <mergeCell ref="C98:C101"/>
+    <mergeCell ref="C154:C157"/>
+    <mergeCell ref="E14:E17"/>
+    <mergeCell ref="A166:A169"/>
+    <mergeCell ref="E102:E105"/>
+    <mergeCell ref="B50:B53"/>
+    <mergeCell ref="A162:A165"/>
+    <mergeCell ref="A18:A21"/>
+    <mergeCell ref="D26:D29"/>
+    <mergeCell ref="A14:A17"/>
+    <mergeCell ref="C18:C21"/>
+    <mergeCell ref="B22:B25"/>
+    <mergeCell ref="D22:D25"/>
+    <mergeCell ref="E18:E21"/>
+    <mergeCell ref="B78:B81"/>
+    <mergeCell ref="F42:F45"/>
+    <mergeCell ref="D78:D81"/>
+    <mergeCell ref="E50:E53"/>
+    <mergeCell ref="D82:D85"/>
+    <mergeCell ref="C86:C89"/>
+    <mergeCell ref="F82:F85"/>
+    <mergeCell ref="C34:C37"/>
+    <mergeCell ref="D54:D57"/>
+    <mergeCell ref="C30:C33"/>
+    <mergeCell ref="E38:E41"/>
+    <mergeCell ref="A54:A57"/>
+    <mergeCell ref="D46:D49"/>
+    <mergeCell ref="C54:C57"/>
+    <mergeCell ref="A74:A77"/>
+    <mergeCell ref="B38:B41"/>
+    <mergeCell ref="F46:F49"/>
+    <mergeCell ref="E74:E77"/>
+    <mergeCell ref="A66:A69"/>
+    <mergeCell ref="D198:D201"/>
+    <mergeCell ref="A90:A93"/>
+    <mergeCell ref="A146:A149"/>
+    <mergeCell ref="F198:F201"/>
+    <mergeCell ref="C146:C149"/>
+    <mergeCell ref="D174:D177"/>
+    <mergeCell ref="F174:F177"/>
+    <mergeCell ref="A178:A181"/>
+    <mergeCell ref="D126:D129"/>
+    <mergeCell ref="C94:C97"/>
+    <mergeCell ref="F126:F129"/>
+    <mergeCell ref="D166:D169"/>
+    <mergeCell ref="E94:E97"/>
+    <mergeCell ref="E90:E93"/>
+    <mergeCell ref="F110:F113"/>
+    <mergeCell ref="D150:D153"/>
+    <mergeCell ref="F150:F153"/>
+    <mergeCell ref="E158:E161"/>
+    <mergeCell ref="B166:B169"/>
+    <mergeCell ref="B118:B121"/>
+    <mergeCell ref="E154:E157"/>
+    <mergeCell ref="E110:E113"/>
+    <mergeCell ref="E130:E133"/>
+    <mergeCell ref="B134:B137"/>
+    <mergeCell ref="E186:E189"/>
+    <mergeCell ref="C106:C109"/>
+    <mergeCell ref="A194:A197"/>
+    <mergeCell ref="A46:A49"/>
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="B158:B161"/>
+    <mergeCell ref="F94:F97"/>
+    <mergeCell ref="C2:C5"/>
+    <mergeCell ref="B6:B9"/>
+    <mergeCell ref="E2:E5"/>
+    <mergeCell ref="B186:B189"/>
+    <mergeCell ref="C82:C85"/>
+    <mergeCell ref="D102:D105"/>
+    <mergeCell ref="B142:B145"/>
+    <mergeCell ref="E174:E177"/>
+    <mergeCell ref="D142:D145"/>
+    <mergeCell ref="A10:A13"/>
+    <mergeCell ref="A22:A25"/>
+    <mergeCell ref="A150:A153"/>
+    <mergeCell ref="E26:E29"/>
+    <mergeCell ref="D98:D101"/>
+    <mergeCell ref="C66:C69"/>
+    <mergeCell ref="A102:A105"/>
+    <mergeCell ref="E66:E69"/>
+    <mergeCell ref="D10:D13"/>
+    <mergeCell ref="B90:B93"/>
+    <mergeCell ref="D50:D53"/>
+    <mergeCell ref="F10:F13"/>
+    <mergeCell ref="A94:A97"/>
+    <mergeCell ref="B122:B125"/>
+    <mergeCell ref="F146:F149"/>
+    <mergeCell ref="E150:E153"/>
+    <mergeCell ref="D178:D181"/>
+    <mergeCell ref="D34:D37"/>
+    <mergeCell ref="F178:F181"/>
+    <mergeCell ref="C42:C45"/>
+    <mergeCell ref="F34:F37"/>
+    <mergeCell ref="A78:A81"/>
+    <mergeCell ref="F74:F77"/>
+    <mergeCell ref="E42:E45"/>
+    <mergeCell ref="B18:B21"/>
+    <mergeCell ref="B106:B109"/>
+    <mergeCell ref="F98:F101"/>
+    <mergeCell ref="C102:C105"/>
+    <mergeCell ref="A34:A37"/>
+    <mergeCell ref="B26:B29"/>
+    <mergeCell ref="F30:F33"/>
+    <mergeCell ref="A30:A33"/>
+    <mergeCell ref="B2:B5"/>
+    <mergeCell ref="D2:D5"/>
+    <mergeCell ref="B42:B45"/>
+    <mergeCell ref="C22:C25"/>
+    <mergeCell ref="E122:E125"/>
+    <mergeCell ref="F18:F21"/>
+    <mergeCell ref="B170:B173"/>
+    <mergeCell ref="E78:E81"/>
+    <mergeCell ref="A174:A177"/>
+    <mergeCell ref="D170:D173"/>
+    <mergeCell ref="B58:B61"/>
+    <mergeCell ref="F2:F5"/>
+    <mergeCell ref="E6:E9"/>
+    <mergeCell ref="C134:C137"/>
+    <mergeCell ref="F22:F25"/>
+    <mergeCell ref="C114:C117"/>
+    <mergeCell ref="A154:A157"/>
+    <mergeCell ref="E30:E33"/>
+    <mergeCell ref="E170:E173"/>
+    <mergeCell ref="E114:E117"/>
+    <mergeCell ref="F102:F105"/>
+    <mergeCell ref="C70:C73"/>
+    <mergeCell ref="E70:E73"/>
+    <mergeCell ref="C46:C49"/>
+    <mergeCell ref="B30:B33"/>
+    <mergeCell ref="C138:C141"/>
+    <mergeCell ref="C178:C181"/>
+    <mergeCell ref="E54:E57"/>
+    <mergeCell ref="D30:D33"/>
+    <mergeCell ref="E178:E181"/>
+    <mergeCell ref="D62:D65"/>
+    <mergeCell ref="D118:D121"/>
+    <mergeCell ref="F62:F65"/>
+    <mergeCell ref="E126:E129"/>
+    <mergeCell ref="C166:C169"/>
+    <mergeCell ref="C126:C129"/>
+    <mergeCell ref="C58:C61"/>
+    <mergeCell ref="E58:E61"/>
+    <mergeCell ref="D90:D93"/>
+    <mergeCell ref="B46:B49"/>
+    <mergeCell ref="B102:B105"/>
+    <mergeCell ref="E138:E141"/>
+    <mergeCell ref="D158:D161"/>
+    <mergeCell ref="B98:B101"/>
+    <mergeCell ref="F114:F117"/>
+    <mergeCell ref="D154:D157"/>
+    <mergeCell ref="C162:C165"/>
+    <mergeCell ref="B130:B133"/>
+    <mergeCell ref="B198:B201"/>
+    <mergeCell ref="D14:D17"/>
+    <mergeCell ref="A106:A109"/>
+    <mergeCell ref="F14:F17"/>
+    <mergeCell ref="B174:B177"/>
+    <mergeCell ref="A38:A41"/>
+    <mergeCell ref="B126:B129"/>
+    <mergeCell ref="D182:D185"/>
+    <mergeCell ref="D38:D41"/>
+    <mergeCell ref="F182:F185"/>
+    <mergeCell ref="A130:A133"/>
+    <mergeCell ref="A82:A85"/>
+    <mergeCell ref="B110:B113"/>
+    <mergeCell ref="E106:E109"/>
+    <mergeCell ref="D110:D113"/>
+    <mergeCell ref="B54:B57"/>
+    <mergeCell ref="E146:E149"/>
+    <mergeCell ref="A58:A61"/>
+    <mergeCell ref="F166:F169"/>
+    <mergeCell ref="E198:E201"/>
+    <mergeCell ref="C74:C77"/>
+    <mergeCell ref="A110:A113"/>
+    <mergeCell ref="F162:F165"/>
+    <mergeCell ref="B94:B97"/>
+    <mergeCell ref="F26:F29"/>
+    <mergeCell ref="C118:C121"/>
+    <mergeCell ref="F154:F157"/>
+    <mergeCell ref="A158:A161"/>
+    <mergeCell ref="D186:D189"/>
+    <mergeCell ref="A6:A9"/>
+    <mergeCell ref="A50:A53"/>
+    <mergeCell ref="C50:C53"/>
+    <mergeCell ref="B82:B85"/>
+    <mergeCell ref="A86:A89"/>
+    <mergeCell ref="F138:F141"/>
+    <mergeCell ref="C142:C145"/>
+    <mergeCell ref="F90:F93"/>
+    <mergeCell ref="E118:E121"/>
+    <mergeCell ref="B10:B13"/>
+    <mergeCell ref="E46:E49"/>
+    <mergeCell ref="D66:D69"/>
+    <mergeCell ref="D106:D109"/>
+    <mergeCell ref="B146:B149"/>
+    <mergeCell ref="F66:F69"/>
+    <mergeCell ref="D18:D21"/>
+    <mergeCell ref="D146:D149"/>
+    <mergeCell ref="E166:E169"/>
+    <mergeCell ref="A26:A29"/>
+    <mergeCell ref="F158:F161"/>
+    <mergeCell ref="B190:B193"/>
+    <mergeCell ref="D194:D197"/>
+    <mergeCell ref="B178:B181"/>
+    <mergeCell ref="E86:E89"/>
+    <mergeCell ref="B34:B37"/>
+    <mergeCell ref="F38:F41"/>
+    <mergeCell ref="A42:A45"/>
+    <mergeCell ref="B74:B77"/>
+    <mergeCell ref="F50:F53"/>
+    <mergeCell ref="E162:E165"/>
+    <mergeCell ref="D130:D133"/>
+    <mergeCell ref="A134:A137"/>
+    <mergeCell ref="B162:B165"/>
+    <mergeCell ref="F130:F133"/>
+    <mergeCell ref="D74:D77"/>
+    <mergeCell ref="E134:E137"/>
+    <mergeCell ref="D138:D141"/>
+    <mergeCell ref="F54:F57"/>
+    <mergeCell ref="C158:C161"/>
+    <mergeCell ref="F190:F193"/>
+    <mergeCell ref="E190:E193"/>
+    <mergeCell ref="B194:B197"/>
+    <mergeCell ref="A182:A185"/>
+    <mergeCell ref="F134:F137"/>
+    <mergeCell ref="E62:E65"/>
+    <mergeCell ref="E22:E25"/>
+    <mergeCell ref="C194:C197"/>
+    <mergeCell ref="C38:C41"/>
+    <mergeCell ref="D58:D61"/>
+    <mergeCell ref="A62:A65"/>
+    <mergeCell ref="F58:F61"/>
+    <mergeCell ref="A122:A125"/>
+    <mergeCell ref="C122:C125"/>
+    <mergeCell ref="C78:C81"/>
+    <mergeCell ref="D42:D45"/>
+    <mergeCell ref="A186:A189"/>
+    <mergeCell ref="C186:C189"/>
+    <mergeCell ref="D94:D97"/>
+    <mergeCell ref="E142:E145"/>
+    <mergeCell ref="E194:E197"/>
+    <mergeCell ref="B150:B153"/>
+    <mergeCell ref="A114:A117"/>
+    <mergeCell ref="A170:A173"/>
+    <mergeCell ref="A70:A73"/>
+    <mergeCell ref="C170:C173"/>
+    <mergeCell ref="F78:F81"/>
+    <mergeCell ref="F118:F121"/>
+    <mergeCell ref="C174:C177"/>
+    <mergeCell ref="F170:F173"/>
+    <mergeCell ref="B138:B141"/>
+    <mergeCell ref="D6:D9"/>
+    <mergeCell ref="C26:C29"/>
+    <mergeCell ref="D190:D193"/>
+    <mergeCell ref="B86:B89"/>
+    <mergeCell ref="A138:A141"/>
+    <mergeCell ref="E82:E85"/>
+    <mergeCell ref="D86:D89"/>
+    <mergeCell ref="F6:F9"/>
+    <mergeCell ref="F86:F89"/>
+    <mergeCell ref="F142:F145"/>
+    <mergeCell ref="C10:C13"/>
+    <mergeCell ref="B62:B65"/>
+    <mergeCell ref="E10:E13"/>
+    <mergeCell ref="B14:B17"/>
+    <mergeCell ref="B70:B73"/>
+    <mergeCell ref="D70:D73"/>
+    <mergeCell ref="E98:E101"/>
+    <mergeCell ref="F70:F73"/>
+    <mergeCell ref="E34:E37"/>
+    <mergeCell ref="B182:B185"/>
+    <mergeCell ref="D134:D137"/>
     <mergeCell ref="C6:C9"/>
     <mergeCell ref="C62:C65"/>
     <mergeCell ref="A98:A101"/>
@@ -3250,282 +3526,6 @@
     <mergeCell ref="B114:B117"/>
     <mergeCell ref="D114:D117"/>
     <mergeCell ref="B154:B157"/>
-    <mergeCell ref="C174:C177"/>
-    <mergeCell ref="F170:F173"/>
-    <mergeCell ref="B138:B141"/>
-    <mergeCell ref="D6:D9"/>
-    <mergeCell ref="C26:C29"/>
-    <mergeCell ref="D190:D193"/>
-    <mergeCell ref="B86:B89"/>
-    <mergeCell ref="A138:A141"/>
-    <mergeCell ref="E82:E85"/>
-    <mergeCell ref="D86:D89"/>
-    <mergeCell ref="F6:F9"/>
-    <mergeCell ref="F86:F89"/>
-    <mergeCell ref="F142:F145"/>
-    <mergeCell ref="C10:C13"/>
-    <mergeCell ref="B62:B65"/>
-    <mergeCell ref="E10:E13"/>
-    <mergeCell ref="B14:B17"/>
-    <mergeCell ref="B70:B73"/>
-    <mergeCell ref="D70:D73"/>
-    <mergeCell ref="E98:E101"/>
-    <mergeCell ref="F70:F73"/>
-    <mergeCell ref="E34:E37"/>
-    <mergeCell ref="B182:B185"/>
-    <mergeCell ref="D134:D137"/>
-    <mergeCell ref="F134:F137"/>
-    <mergeCell ref="E62:E65"/>
-    <mergeCell ref="E22:E25"/>
-    <mergeCell ref="C194:C197"/>
-    <mergeCell ref="C38:C41"/>
-    <mergeCell ref="D58:D61"/>
-    <mergeCell ref="A62:A65"/>
-    <mergeCell ref="F58:F61"/>
-    <mergeCell ref="A122:A125"/>
-    <mergeCell ref="C122:C125"/>
-    <mergeCell ref="C78:C81"/>
-    <mergeCell ref="D42:D45"/>
-    <mergeCell ref="A186:A189"/>
-    <mergeCell ref="C186:C189"/>
-    <mergeCell ref="D94:D97"/>
-    <mergeCell ref="E142:E145"/>
-    <mergeCell ref="E194:E197"/>
-    <mergeCell ref="B150:B153"/>
-    <mergeCell ref="A114:A117"/>
-    <mergeCell ref="A170:A173"/>
-    <mergeCell ref="A70:A73"/>
-    <mergeCell ref="C170:C173"/>
-    <mergeCell ref="F78:F81"/>
-    <mergeCell ref="F118:F121"/>
-    <mergeCell ref="F158:F161"/>
-    <mergeCell ref="B190:B193"/>
-    <mergeCell ref="D194:D197"/>
-    <mergeCell ref="B178:B181"/>
-    <mergeCell ref="E86:E89"/>
-    <mergeCell ref="B34:B37"/>
-    <mergeCell ref="F38:F41"/>
-    <mergeCell ref="A42:A45"/>
-    <mergeCell ref="B74:B77"/>
-    <mergeCell ref="F50:F53"/>
-    <mergeCell ref="E162:E165"/>
-    <mergeCell ref="D130:D133"/>
-    <mergeCell ref="A134:A137"/>
-    <mergeCell ref="B162:B165"/>
-    <mergeCell ref="F130:F133"/>
-    <mergeCell ref="D74:D77"/>
-    <mergeCell ref="E134:E137"/>
-    <mergeCell ref="D138:D141"/>
-    <mergeCell ref="F54:F57"/>
-    <mergeCell ref="C158:C161"/>
-    <mergeCell ref="F26:F29"/>
-    <mergeCell ref="C118:C121"/>
-    <mergeCell ref="F154:F157"/>
-    <mergeCell ref="A158:A161"/>
-    <mergeCell ref="D186:D189"/>
-    <mergeCell ref="A6:A9"/>
-    <mergeCell ref="A50:A53"/>
-    <mergeCell ref="C50:C53"/>
-    <mergeCell ref="B82:B85"/>
-    <mergeCell ref="A86:A89"/>
-    <mergeCell ref="F138:F141"/>
-    <mergeCell ref="C142:C145"/>
-    <mergeCell ref="F90:F93"/>
-    <mergeCell ref="E118:E121"/>
-    <mergeCell ref="B10:B13"/>
-    <mergeCell ref="E46:E49"/>
-    <mergeCell ref="D66:D69"/>
-    <mergeCell ref="D106:D109"/>
-    <mergeCell ref="B146:B149"/>
-    <mergeCell ref="F66:F69"/>
-    <mergeCell ref="D18:D21"/>
-    <mergeCell ref="D146:D149"/>
-    <mergeCell ref="E166:E169"/>
-    <mergeCell ref="A26:A29"/>
-    <mergeCell ref="B198:B201"/>
-    <mergeCell ref="D14:D17"/>
-    <mergeCell ref="A106:A109"/>
-    <mergeCell ref="F14:F17"/>
-    <mergeCell ref="B174:B177"/>
-    <mergeCell ref="A38:A41"/>
-    <mergeCell ref="B126:B129"/>
-    <mergeCell ref="D182:D185"/>
-    <mergeCell ref="D38:D41"/>
-    <mergeCell ref="F182:F185"/>
-    <mergeCell ref="A130:A133"/>
-    <mergeCell ref="A82:A85"/>
-    <mergeCell ref="B110:B113"/>
-    <mergeCell ref="E106:E109"/>
-    <mergeCell ref="D110:D113"/>
-    <mergeCell ref="B54:B57"/>
-    <mergeCell ref="E146:E149"/>
-    <mergeCell ref="A58:A61"/>
-    <mergeCell ref="F166:F169"/>
-    <mergeCell ref="E198:E201"/>
-    <mergeCell ref="C74:C77"/>
-    <mergeCell ref="A110:A113"/>
-    <mergeCell ref="F162:F165"/>
-    <mergeCell ref="B94:B97"/>
-    <mergeCell ref="F190:F193"/>
-    <mergeCell ref="B30:B33"/>
-    <mergeCell ref="C138:C141"/>
-    <mergeCell ref="C178:C181"/>
-    <mergeCell ref="E54:E57"/>
-    <mergeCell ref="D30:D33"/>
-    <mergeCell ref="E178:E181"/>
-    <mergeCell ref="D62:D65"/>
-    <mergeCell ref="D118:D121"/>
-    <mergeCell ref="F62:F65"/>
-    <mergeCell ref="E126:E129"/>
-    <mergeCell ref="C166:C169"/>
-    <mergeCell ref="C126:C129"/>
-    <mergeCell ref="C58:C61"/>
-    <mergeCell ref="E58:E61"/>
-    <mergeCell ref="D90:D93"/>
-    <mergeCell ref="B46:B49"/>
-    <mergeCell ref="B102:B105"/>
-    <mergeCell ref="E138:E141"/>
-    <mergeCell ref="E190:E193"/>
-    <mergeCell ref="D158:D161"/>
-    <mergeCell ref="B98:B101"/>
-    <mergeCell ref="F114:F117"/>
-    <mergeCell ref="D154:D157"/>
-    <mergeCell ref="B2:B5"/>
-    <mergeCell ref="D2:D5"/>
-    <mergeCell ref="B42:B45"/>
-    <mergeCell ref="C22:C25"/>
-    <mergeCell ref="E122:E125"/>
-    <mergeCell ref="F18:F21"/>
-    <mergeCell ref="B170:B173"/>
-    <mergeCell ref="E78:E81"/>
-    <mergeCell ref="A174:A177"/>
-    <mergeCell ref="D170:D173"/>
-    <mergeCell ref="B58:B61"/>
-    <mergeCell ref="F2:F5"/>
-    <mergeCell ref="E6:E9"/>
-    <mergeCell ref="C134:C137"/>
-    <mergeCell ref="F22:F25"/>
-    <mergeCell ref="C114:C117"/>
-    <mergeCell ref="A154:A157"/>
-    <mergeCell ref="E30:E33"/>
-    <mergeCell ref="E170:E173"/>
-    <mergeCell ref="E114:E117"/>
-    <mergeCell ref="F102:F105"/>
-    <mergeCell ref="C70:C73"/>
-    <mergeCell ref="E70:E73"/>
-    <mergeCell ref="C46:C49"/>
-    <mergeCell ref="B194:B197"/>
-    <mergeCell ref="D10:D13"/>
-    <mergeCell ref="B90:B93"/>
-    <mergeCell ref="D50:D53"/>
-    <mergeCell ref="F10:F13"/>
-    <mergeCell ref="A94:A97"/>
-    <mergeCell ref="B122:B125"/>
-    <mergeCell ref="F146:F149"/>
-    <mergeCell ref="E150:E153"/>
-    <mergeCell ref="D178:D181"/>
-    <mergeCell ref="D34:D37"/>
-    <mergeCell ref="A182:A185"/>
-    <mergeCell ref="F178:F181"/>
-    <mergeCell ref="C42:C45"/>
-    <mergeCell ref="F34:F37"/>
-    <mergeCell ref="A78:A81"/>
-    <mergeCell ref="F74:F77"/>
-    <mergeCell ref="E42:E45"/>
-    <mergeCell ref="B18:B21"/>
-    <mergeCell ref="B106:B109"/>
-    <mergeCell ref="E186:E189"/>
-    <mergeCell ref="C106:C109"/>
-    <mergeCell ref="A194:A197"/>
-    <mergeCell ref="A46:A49"/>
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="B158:B161"/>
-    <mergeCell ref="F94:F97"/>
-    <mergeCell ref="C2:C5"/>
-    <mergeCell ref="B6:B9"/>
-    <mergeCell ref="E2:E5"/>
-    <mergeCell ref="B186:B189"/>
-    <mergeCell ref="C82:C85"/>
-    <mergeCell ref="D102:D105"/>
-    <mergeCell ref="B142:B145"/>
-    <mergeCell ref="E174:E177"/>
-    <mergeCell ref="D142:D145"/>
-    <mergeCell ref="A10:A13"/>
-    <mergeCell ref="A22:A25"/>
-    <mergeCell ref="A150:A153"/>
-    <mergeCell ref="E26:E29"/>
-    <mergeCell ref="D98:D101"/>
-    <mergeCell ref="C66:C69"/>
-    <mergeCell ref="A102:A105"/>
-    <mergeCell ref="E66:E69"/>
-    <mergeCell ref="F98:F101"/>
-    <mergeCell ref="C102:C105"/>
-    <mergeCell ref="A34:A37"/>
-    <mergeCell ref="B26:B29"/>
-    <mergeCell ref="D198:D201"/>
-    <mergeCell ref="A90:A93"/>
-    <mergeCell ref="A146:A149"/>
-    <mergeCell ref="F198:F201"/>
-    <mergeCell ref="C146:C149"/>
-    <mergeCell ref="D174:D177"/>
-    <mergeCell ref="F174:F177"/>
-    <mergeCell ref="A178:A181"/>
-    <mergeCell ref="D126:D129"/>
-    <mergeCell ref="C94:C97"/>
-    <mergeCell ref="F126:F129"/>
-    <mergeCell ref="D166:D169"/>
-    <mergeCell ref="E94:E97"/>
-    <mergeCell ref="E90:E93"/>
-    <mergeCell ref="F110:F113"/>
-    <mergeCell ref="D150:D153"/>
-    <mergeCell ref="F150:F153"/>
-    <mergeCell ref="E158:E161"/>
-    <mergeCell ref="B166:B169"/>
-    <mergeCell ref="B118:B121"/>
-    <mergeCell ref="E154:E157"/>
-    <mergeCell ref="E110:E113"/>
-    <mergeCell ref="E130:E133"/>
-    <mergeCell ref="B134:B137"/>
-    <mergeCell ref="F30:F33"/>
-    <mergeCell ref="A30:A33"/>
-    <mergeCell ref="C162:C165"/>
-    <mergeCell ref="B130:B133"/>
-    <mergeCell ref="C30:C33"/>
-    <mergeCell ref="E38:E41"/>
-    <mergeCell ref="A54:A57"/>
-    <mergeCell ref="D46:D49"/>
-    <mergeCell ref="C54:C57"/>
-    <mergeCell ref="A74:A77"/>
-    <mergeCell ref="B38:B41"/>
-    <mergeCell ref="F46:F49"/>
-    <mergeCell ref="E74:E77"/>
-    <mergeCell ref="B78:B81"/>
-    <mergeCell ref="F42:F45"/>
-    <mergeCell ref="D78:D81"/>
-    <mergeCell ref="E50:E53"/>
-    <mergeCell ref="D82:D85"/>
-    <mergeCell ref="C86:C89"/>
-    <mergeCell ref="F82:F85"/>
-    <mergeCell ref="C34:C37"/>
-    <mergeCell ref="D54:D57"/>
-    <mergeCell ref="A66:A69"/>
-    <mergeCell ref="A118:A121"/>
-    <mergeCell ref="C14:C17"/>
-    <mergeCell ref="B66:B69"/>
-    <mergeCell ref="C98:C101"/>
-    <mergeCell ref="C154:C157"/>
-    <mergeCell ref="E14:E17"/>
-    <mergeCell ref="A166:A169"/>
-    <mergeCell ref="E102:E105"/>
-    <mergeCell ref="B50:B53"/>
-    <mergeCell ref="A162:A165"/>
-    <mergeCell ref="A18:A21"/>
-    <mergeCell ref="D26:D29"/>
-    <mergeCell ref="A14:A17"/>
-    <mergeCell ref="C18:C21"/>
-    <mergeCell ref="B22:B25"/>
-    <mergeCell ref="D22:D25"/>
-    <mergeCell ref="E18:E21"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Assignment 1 test cases and remove temp file
Replace the binary workbook 'Assignment 1 - Test cases.xlsx' with an updated version and delete the temporary autosave file '~$Assignment 1 - Test cases.xlsx'. Cleans up the repo and updates the test cases spreadsheet.
</commit_message>
<xml_diff>
--- a/Assignment 1 - Test cases.xlsx
+++ b/Assignment 1 - Test cases.xlsx
@@ -700,13 +700,13 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
@@ -1040,7 +1040,7 @@
       <c r="E2" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="F2" s="8" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1081,10 +1081,10 @@
       <c r="D6" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E6" s="8" t="s">
+      <c r="E6" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="F6" s="5" t="s">
+      <c r="F6" s="8" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1125,10 +1125,10 @@
       <c r="D10" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E10" s="8" t="s">
+      <c r="E10" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="F10" s="5" t="s">
+      <c r="F10" s="8" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1169,10 +1169,10 @@
       <c r="D14" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="E14" s="8" t="s">
+      <c r="E14" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="F14" s="5" t="s">
+      <c r="F14" s="8" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1213,10 +1213,10 @@
       <c r="D18" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="E18" s="8" t="s">
+      <c r="E18" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="F18" s="5" t="s">
+      <c r="F18" s="8" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1257,10 +1257,10 @@
       <c r="D22" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="E22" s="8" t="s">
+      <c r="E22" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="F22" s="5" t="s">
+      <c r="F22" s="8" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1301,10 +1301,10 @@
       <c r="D26" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="E26" s="8" t="s">
+      <c r="E26" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="F26" s="5" t="s">
+      <c r="F26" s="8" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1345,10 +1345,10 @@
       <c r="D30" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="E30" s="8" t="s">
+      <c r="E30" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="F30" s="5" t="s">
+      <c r="F30" s="8" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1389,10 +1389,10 @@
       <c r="D34" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="E34" s="8" t="s">
+      <c r="E34" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="F34" s="5" t="s">
+      <c r="F34" s="8" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1433,10 +1433,10 @@
       <c r="D38" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="E38" s="8" t="s">
+      <c r="E38" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="F38" s="5" t="s">
+      <c r="F38" s="8" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1477,10 +1477,10 @@
       <c r="D42" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="E42" s="8" t="s">
+      <c r="E42" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="F42" s="5" t="s">
+      <c r="F42" s="8" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1521,10 +1521,10 @@
       <c r="D46" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="E46" s="8" t="s">
+      <c r="E46" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="F46" s="5" t="s">
+      <c r="F46" s="8" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1565,10 +1565,10 @@
       <c r="D50" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="E50" s="8" t="s">
+      <c r="E50" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="F50" s="5" t="s">
+      <c r="F50" s="8" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1609,10 +1609,10 @@
       <c r="D54" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="E54" s="8" t="s">
+      <c r="E54" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="F54" s="5" t="s">
+      <c r="F54" s="8" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1653,10 +1653,10 @@
       <c r="D58" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="E58" s="8" t="s">
+      <c r="E58" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="F58" s="5" t="s">
+      <c r="F58" s="8" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1697,10 +1697,10 @@
       <c r="D62" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="E62" s="8" t="s">
+      <c r="E62" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="F62" s="5" t="s">
+      <c r="F62" s="8" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1741,10 +1741,10 @@
       <c r="D66" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="E66" s="8" t="s">
+      <c r="E66" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="F66" s="5" t="s">
+      <c r="F66" s="8" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1785,10 +1785,10 @@
       <c r="D70" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="E70" s="8" t="s">
+      <c r="E70" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="F70" s="5" t="s">
+      <c r="F70" s="8" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1829,10 +1829,10 @@
       <c r="D74" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="E74" s="8" t="s">
+      <c r="E74" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="F74" s="5" t="s">
+      <c r="F74" s="8" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1873,10 +1873,10 @@
       <c r="D78" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="E78" s="8" t="s">
+      <c r="E78" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="F78" s="5" t="s">
+      <c r="F78" s="8" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1917,10 +1917,10 @@
       <c r="D82" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="E82" s="8" t="s">
+      <c r="E82" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="F82" s="5" t="s">
+      <c r="F82" s="8" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1961,10 +1961,10 @@
       <c r="D86" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="E86" s="8" t="s">
+      <c r="E86" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="F86" s="5" t="s">
+      <c r="F86" s="8" t="s">
         <v>13</v>
       </c>
     </row>
@@ -2005,10 +2005,10 @@
       <c r="D90" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="E90" s="8" t="s">
+      <c r="E90" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="F90" s="5" t="s">
+      <c r="F90" s="8" t="s">
         <v>13</v>
       </c>
     </row>
@@ -2049,10 +2049,10 @@
       <c r="D94" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="E94" s="8" t="s">
+      <c r="E94" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="F94" s="5" t="s">
+      <c r="F94" s="8" t="s">
         <v>13</v>
       </c>
     </row>
@@ -2093,10 +2093,10 @@
       <c r="D98" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="E98" s="8" t="s">
+      <c r="E98" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="F98" s="5" t="s">
+      <c r="F98" s="8" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2137,10 +2137,10 @@
       <c r="D102" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="E102" s="8" t="s">
+      <c r="E102" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="F102" s="5" t="s">
+      <c r="F102" s="8" t="s">
         <v>13</v>
       </c>
     </row>
@@ -2181,10 +2181,10 @@
       <c r="D106" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="E106" s="8" t="s">
+      <c r="E106" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="F106" s="5" t="s">
+      <c r="F106" s="8" t="s">
         <v>13</v>
       </c>
     </row>
@@ -2225,10 +2225,10 @@
       <c r="D110" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="E110" s="8" t="s">
+      <c r="E110" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="F110" s="5" t="s">
+      <c r="F110" s="8" t="s">
         <v>13</v>
       </c>
     </row>
@@ -2269,10 +2269,10 @@
       <c r="D114" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="E114" s="8" t="s">
+      <c r="E114" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="F114" s="5" t="s">
+      <c r="F114" s="8" t="s">
         <v>13</v>
       </c>
     </row>
@@ -2313,10 +2313,10 @@
       <c r="D118" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="E118" s="8" t="s">
+      <c r="E118" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="F118" s="5" t="s">
+      <c r="F118" s="8" t="s">
         <v>13</v>
       </c>
     </row>
@@ -2357,10 +2357,10 @@
       <c r="D122" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="E122" s="8" t="s">
+      <c r="E122" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="F122" s="5" t="s">
+      <c r="F122" s="8" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2401,10 +2401,10 @@
       <c r="D126" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="E126" s="8" t="s">
+      <c r="E126" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="F126" s="5" t="s">
+      <c r="F126" s="8" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2445,10 +2445,10 @@
       <c r="D130" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="E130" s="8" t="s">
+      <c r="E130" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="F130" s="5" t="s">
+      <c r="F130" s="8" t="s">
         <v>13</v>
       </c>
     </row>
@@ -2489,10 +2489,10 @@
       <c r="D134" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="E134" s="8" t="s">
+      <c r="E134" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="F134" s="5" t="s">
+      <c r="F134" s="8" t="s">
         <v>13</v>
       </c>
     </row>
@@ -2533,10 +2533,10 @@
       <c r="D138" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="E138" s="8" t="s">
+      <c r="E138" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="F138" s="5" t="s">
+      <c r="F138" s="8" t="s">
         <v>13</v>
       </c>
     </row>
@@ -2577,10 +2577,10 @@
       <c r="D142" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="E142" s="8" t="s">
+      <c r="E142" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="F142" s="5" t="s">
+      <c r="F142" s="8" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2621,10 +2621,10 @@
       <c r="D146" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="E146" s="8" t="s">
+      <c r="E146" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="F146" s="5" t="s">
+      <c r="F146" s="8" t="s">
         <v>13</v>
       </c>
     </row>
@@ -2665,10 +2665,10 @@
       <c r="D150" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="E150" s="8" t="s">
+      <c r="E150" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="F150" s="5" t="s">
+      <c r="F150" s="8" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2709,10 +2709,10 @@
       <c r="D154" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="E154" s="8" t="s">
+      <c r="E154" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="F154" s="5" t="s">
+      <c r="F154" s="8" t="s">
         <v>13</v>
       </c>
     </row>
@@ -2753,10 +2753,10 @@
       <c r="D158" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="E158" s="8" t="s">
+      <c r="E158" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="F158" s="5" t="s">
+      <c r="F158" s="8" t="s">
         <v>13</v>
       </c>
     </row>
@@ -2797,10 +2797,10 @@
       <c r="D162" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="E162" s="8" t="s">
+      <c r="E162" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="F162" s="5" t="s">
+      <c r="F162" s="8" t="s">
         <v>13</v>
       </c>
     </row>
@@ -2841,10 +2841,10 @@
       <c r="D166" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="E166" s="8" t="s">
+      <c r="E166" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="F166" s="5" t="s">
+      <c r="F166" s="8" t="s">
         <v>13</v>
       </c>
     </row>
@@ -2885,10 +2885,10 @@
       <c r="D170" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="E170" s="8" t="s">
+      <c r="E170" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="F170" s="5" t="s">
+      <c r="F170" s="8" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2929,10 +2929,10 @@
       <c r="D174" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="E174" s="8" t="s">
+      <c r="E174" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="F174" s="5" t="s">
+      <c r="F174" s="8" t="s">
         <v>13</v>
       </c>
     </row>
@@ -2973,10 +2973,10 @@
       <c r="D178" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="E178" s="8" t="s">
+      <c r="E178" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="F178" s="5" t="s">
+      <c r="F178" s="8" t="s">
         <v>10</v>
       </c>
     </row>
@@ -3017,10 +3017,10 @@
       <c r="D182" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="E182" s="8" t="s">
+      <c r="E182" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="F182" s="5" t="s">
+      <c r="F182" s="8" t="s">
         <v>10</v>
       </c>
     </row>
@@ -3061,10 +3061,10 @@
       <c r="D186" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="E186" s="8" t="s">
+      <c r="E186" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="F186" s="5" t="s">
+      <c r="F186" s="8" t="s">
         <v>13</v>
       </c>
     </row>
@@ -3105,10 +3105,10 @@
       <c r="D190" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="E190" s="8" t="s">
+      <c r="E190" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="F190" s="5" t="s">
+      <c r="F190" s="8" t="s">
         <v>10</v>
       </c>
     </row>
@@ -3149,10 +3149,10 @@
       <c r="D194" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="E194" s="8" t="s">
+      <c r="E194" s="5" t="s">
         <v>125</v>
       </c>
-      <c r="F194" s="5" t="s">
+      <c r="F194" s="8" t="s">
         <v>10</v>
       </c>
     </row>
@@ -3193,10 +3193,10 @@
       <c r="D198" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="E198" s="8" t="s">
+      <c r="E198" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="F198" s="5" t="s">
+      <c r="F198" s="8" t="s">
         <v>10</v>
       </c>
     </row>
@@ -3226,42 +3226,244 @@
     </row>
   </sheetData>
   <mergeCells count="300">
-    <mergeCell ref="A118:A121"/>
-    <mergeCell ref="C14:C17"/>
-    <mergeCell ref="B66:B69"/>
-    <mergeCell ref="C98:C101"/>
-    <mergeCell ref="C154:C157"/>
-    <mergeCell ref="E14:E17"/>
-    <mergeCell ref="A166:A169"/>
-    <mergeCell ref="E102:E105"/>
-    <mergeCell ref="B50:B53"/>
-    <mergeCell ref="A162:A165"/>
-    <mergeCell ref="A18:A21"/>
-    <mergeCell ref="D26:D29"/>
-    <mergeCell ref="A14:A17"/>
-    <mergeCell ref="C18:C21"/>
-    <mergeCell ref="B22:B25"/>
-    <mergeCell ref="D22:D25"/>
-    <mergeCell ref="E18:E21"/>
-    <mergeCell ref="B78:B81"/>
-    <mergeCell ref="F42:F45"/>
-    <mergeCell ref="D78:D81"/>
-    <mergeCell ref="E50:E53"/>
-    <mergeCell ref="D82:D85"/>
-    <mergeCell ref="C86:C89"/>
-    <mergeCell ref="F82:F85"/>
-    <mergeCell ref="C34:C37"/>
-    <mergeCell ref="D54:D57"/>
-    <mergeCell ref="C30:C33"/>
-    <mergeCell ref="E38:E41"/>
-    <mergeCell ref="A54:A57"/>
-    <mergeCell ref="D46:D49"/>
-    <mergeCell ref="C54:C57"/>
-    <mergeCell ref="A74:A77"/>
-    <mergeCell ref="B38:B41"/>
-    <mergeCell ref="F46:F49"/>
-    <mergeCell ref="E74:E77"/>
-    <mergeCell ref="A66:A69"/>
+    <mergeCell ref="F194:F197"/>
+    <mergeCell ref="A198:A201"/>
+    <mergeCell ref="C198:C201"/>
+    <mergeCell ref="D122:D125"/>
+    <mergeCell ref="C90:C93"/>
+    <mergeCell ref="A126:A129"/>
+    <mergeCell ref="D162:D165"/>
+    <mergeCell ref="C130:C133"/>
+    <mergeCell ref="F122:F125"/>
+    <mergeCell ref="C182:C185"/>
+    <mergeCell ref="A142:A145"/>
+    <mergeCell ref="E182:E185"/>
+    <mergeCell ref="C110:C113"/>
+    <mergeCell ref="F106:F109"/>
+    <mergeCell ref="A190:A193"/>
+    <mergeCell ref="C150:C153"/>
+    <mergeCell ref="F186:F189"/>
+    <mergeCell ref="C190:C193"/>
+    <mergeCell ref="B114:B117"/>
+    <mergeCell ref="D114:D117"/>
+    <mergeCell ref="B154:B157"/>
+    <mergeCell ref="D6:D9"/>
+    <mergeCell ref="C26:C29"/>
+    <mergeCell ref="D190:D193"/>
+    <mergeCell ref="B86:B89"/>
+    <mergeCell ref="A138:A141"/>
+    <mergeCell ref="E82:E85"/>
+    <mergeCell ref="D86:D89"/>
+    <mergeCell ref="F6:F9"/>
+    <mergeCell ref="F86:F89"/>
+    <mergeCell ref="F142:F145"/>
+    <mergeCell ref="C10:C13"/>
+    <mergeCell ref="B62:B65"/>
+    <mergeCell ref="E10:E13"/>
+    <mergeCell ref="B14:B17"/>
+    <mergeCell ref="B70:B73"/>
+    <mergeCell ref="D70:D73"/>
+    <mergeCell ref="E98:E101"/>
+    <mergeCell ref="F70:F73"/>
+    <mergeCell ref="E34:E37"/>
+    <mergeCell ref="B182:B185"/>
+    <mergeCell ref="D134:D137"/>
+    <mergeCell ref="C6:C9"/>
+    <mergeCell ref="C62:C65"/>
+    <mergeCell ref="A98:A101"/>
+    <mergeCell ref="E22:E25"/>
+    <mergeCell ref="C194:C197"/>
+    <mergeCell ref="C38:C41"/>
+    <mergeCell ref="D58:D61"/>
+    <mergeCell ref="A62:A65"/>
+    <mergeCell ref="F58:F61"/>
+    <mergeCell ref="A122:A125"/>
+    <mergeCell ref="C122:C125"/>
+    <mergeCell ref="C78:C81"/>
+    <mergeCell ref="D42:D45"/>
+    <mergeCell ref="A186:A189"/>
+    <mergeCell ref="C186:C189"/>
+    <mergeCell ref="D94:D97"/>
+    <mergeCell ref="E142:E145"/>
+    <mergeCell ref="E194:E197"/>
+    <mergeCell ref="B150:B153"/>
+    <mergeCell ref="A114:A117"/>
+    <mergeCell ref="A170:A173"/>
+    <mergeCell ref="A70:A73"/>
+    <mergeCell ref="C170:C173"/>
+    <mergeCell ref="F78:F81"/>
+    <mergeCell ref="F118:F121"/>
+    <mergeCell ref="C174:C177"/>
+    <mergeCell ref="F170:F173"/>
+    <mergeCell ref="B190:B193"/>
+    <mergeCell ref="D194:D197"/>
+    <mergeCell ref="B178:B181"/>
+    <mergeCell ref="E86:E89"/>
+    <mergeCell ref="B34:B37"/>
+    <mergeCell ref="F38:F41"/>
+    <mergeCell ref="A42:A45"/>
+    <mergeCell ref="B74:B77"/>
+    <mergeCell ref="F50:F53"/>
+    <mergeCell ref="E162:E165"/>
+    <mergeCell ref="D130:D133"/>
+    <mergeCell ref="A134:A137"/>
+    <mergeCell ref="B162:B165"/>
+    <mergeCell ref="F130:F133"/>
+    <mergeCell ref="D74:D77"/>
+    <mergeCell ref="E134:E137"/>
+    <mergeCell ref="D138:D141"/>
+    <mergeCell ref="F54:F57"/>
+    <mergeCell ref="C158:C161"/>
+    <mergeCell ref="F190:F193"/>
+    <mergeCell ref="E190:E193"/>
+    <mergeCell ref="B194:B197"/>
+    <mergeCell ref="A182:A185"/>
+    <mergeCell ref="F134:F137"/>
+    <mergeCell ref="F26:F29"/>
+    <mergeCell ref="C118:C121"/>
+    <mergeCell ref="F154:F157"/>
+    <mergeCell ref="A158:A161"/>
+    <mergeCell ref="D186:D189"/>
+    <mergeCell ref="A6:A9"/>
+    <mergeCell ref="A50:A53"/>
+    <mergeCell ref="C50:C53"/>
+    <mergeCell ref="B82:B85"/>
+    <mergeCell ref="A86:A89"/>
+    <mergeCell ref="F138:F141"/>
+    <mergeCell ref="C142:C145"/>
+    <mergeCell ref="F90:F93"/>
+    <mergeCell ref="E118:E121"/>
+    <mergeCell ref="B10:B13"/>
+    <mergeCell ref="E46:E49"/>
+    <mergeCell ref="D66:D69"/>
+    <mergeCell ref="D106:D109"/>
+    <mergeCell ref="B146:B149"/>
+    <mergeCell ref="F66:F69"/>
+    <mergeCell ref="D18:D21"/>
+    <mergeCell ref="D146:D149"/>
+    <mergeCell ref="E166:E169"/>
+    <mergeCell ref="A26:A29"/>
+    <mergeCell ref="B198:B201"/>
+    <mergeCell ref="D14:D17"/>
+    <mergeCell ref="A106:A109"/>
+    <mergeCell ref="F14:F17"/>
+    <mergeCell ref="B174:B177"/>
+    <mergeCell ref="A38:A41"/>
+    <mergeCell ref="B126:B129"/>
+    <mergeCell ref="D182:D185"/>
+    <mergeCell ref="D38:D41"/>
+    <mergeCell ref="F182:F185"/>
+    <mergeCell ref="A130:A133"/>
+    <mergeCell ref="A82:A85"/>
+    <mergeCell ref="B110:B113"/>
+    <mergeCell ref="E106:E109"/>
+    <mergeCell ref="D110:D113"/>
+    <mergeCell ref="B54:B57"/>
+    <mergeCell ref="E146:E149"/>
+    <mergeCell ref="A58:A61"/>
+    <mergeCell ref="F166:F169"/>
+    <mergeCell ref="E198:E201"/>
+    <mergeCell ref="C74:C77"/>
+    <mergeCell ref="A110:A113"/>
+    <mergeCell ref="F162:F165"/>
+    <mergeCell ref="B94:B97"/>
+    <mergeCell ref="B46:B49"/>
+    <mergeCell ref="B102:B105"/>
+    <mergeCell ref="E138:E141"/>
+    <mergeCell ref="D158:D161"/>
+    <mergeCell ref="B98:B101"/>
+    <mergeCell ref="F114:F117"/>
+    <mergeCell ref="D154:D157"/>
+    <mergeCell ref="C162:C165"/>
+    <mergeCell ref="B130:B133"/>
+    <mergeCell ref="F158:F161"/>
+    <mergeCell ref="E62:E65"/>
+    <mergeCell ref="B138:B141"/>
+    <mergeCell ref="C178:C181"/>
+    <mergeCell ref="E54:E57"/>
+    <mergeCell ref="D30:D33"/>
+    <mergeCell ref="E178:E181"/>
+    <mergeCell ref="D62:D65"/>
+    <mergeCell ref="D118:D121"/>
+    <mergeCell ref="F62:F65"/>
+    <mergeCell ref="E126:E129"/>
+    <mergeCell ref="C166:C169"/>
+    <mergeCell ref="C126:C129"/>
+    <mergeCell ref="C58:C61"/>
+    <mergeCell ref="E58:E61"/>
+    <mergeCell ref="D90:D93"/>
+    <mergeCell ref="B2:B5"/>
+    <mergeCell ref="D2:D5"/>
+    <mergeCell ref="B42:B45"/>
+    <mergeCell ref="C22:C25"/>
+    <mergeCell ref="E122:E125"/>
+    <mergeCell ref="F18:F21"/>
+    <mergeCell ref="B170:B173"/>
+    <mergeCell ref="E78:E81"/>
+    <mergeCell ref="A174:A177"/>
+    <mergeCell ref="D170:D173"/>
+    <mergeCell ref="B58:B61"/>
+    <mergeCell ref="F2:F5"/>
+    <mergeCell ref="E6:E9"/>
+    <mergeCell ref="C134:C137"/>
+    <mergeCell ref="F22:F25"/>
+    <mergeCell ref="C114:C117"/>
+    <mergeCell ref="A154:A157"/>
+    <mergeCell ref="E30:E33"/>
+    <mergeCell ref="E170:E173"/>
+    <mergeCell ref="E114:E117"/>
+    <mergeCell ref="F102:F105"/>
+    <mergeCell ref="C70:C73"/>
+    <mergeCell ref="E70:E73"/>
+    <mergeCell ref="C46:C49"/>
+    <mergeCell ref="D10:D13"/>
+    <mergeCell ref="B90:B93"/>
+    <mergeCell ref="D50:D53"/>
+    <mergeCell ref="F10:F13"/>
+    <mergeCell ref="A94:A97"/>
+    <mergeCell ref="B122:B125"/>
+    <mergeCell ref="F146:F149"/>
+    <mergeCell ref="E150:E153"/>
+    <mergeCell ref="D178:D181"/>
+    <mergeCell ref="D34:D37"/>
+    <mergeCell ref="F178:F181"/>
+    <mergeCell ref="C42:C45"/>
+    <mergeCell ref="F34:F37"/>
+    <mergeCell ref="A78:A81"/>
+    <mergeCell ref="F74:F77"/>
+    <mergeCell ref="E42:E45"/>
+    <mergeCell ref="B18:B21"/>
+    <mergeCell ref="B106:B109"/>
+    <mergeCell ref="F98:F101"/>
+    <mergeCell ref="C102:C105"/>
+    <mergeCell ref="A34:A37"/>
+    <mergeCell ref="B26:B29"/>
+    <mergeCell ref="F30:F33"/>
+    <mergeCell ref="A30:A33"/>
+    <mergeCell ref="E186:E189"/>
+    <mergeCell ref="C106:C109"/>
+    <mergeCell ref="A194:A197"/>
+    <mergeCell ref="A46:A49"/>
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="B158:B161"/>
+    <mergeCell ref="F94:F97"/>
+    <mergeCell ref="C2:C5"/>
+    <mergeCell ref="B6:B9"/>
+    <mergeCell ref="E2:E5"/>
+    <mergeCell ref="B186:B189"/>
+    <mergeCell ref="C82:C85"/>
+    <mergeCell ref="D102:D105"/>
+    <mergeCell ref="B142:B145"/>
+    <mergeCell ref="E174:E177"/>
+    <mergeCell ref="D142:D145"/>
+    <mergeCell ref="A10:A13"/>
+    <mergeCell ref="A22:A25"/>
+    <mergeCell ref="A150:A153"/>
+    <mergeCell ref="E26:E29"/>
+    <mergeCell ref="D98:D101"/>
+    <mergeCell ref="C66:C69"/>
+    <mergeCell ref="A102:A105"/>
+    <mergeCell ref="E66:E69"/>
     <mergeCell ref="D198:D201"/>
     <mergeCell ref="A90:A93"/>
     <mergeCell ref="A146:A149"/>
@@ -3286,246 +3488,44 @@
     <mergeCell ref="E110:E113"/>
     <mergeCell ref="E130:E133"/>
     <mergeCell ref="B134:B137"/>
-    <mergeCell ref="E186:E189"/>
-    <mergeCell ref="C106:C109"/>
-    <mergeCell ref="A194:A197"/>
-    <mergeCell ref="A46:A49"/>
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="B158:B161"/>
-    <mergeCell ref="F94:F97"/>
-    <mergeCell ref="C2:C5"/>
-    <mergeCell ref="B6:B9"/>
-    <mergeCell ref="E2:E5"/>
-    <mergeCell ref="B186:B189"/>
-    <mergeCell ref="C82:C85"/>
-    <mergeCell ref="D102:D105"/>
-    <mergeCell ref="B142:B145"/>
-    <mergeCell ref="E174:E177"/>
-    <mergeCell ref="D142:D145"/>
-    <mergeCell ref="A10:A13"/>
-    <mergeCell ref="A22:A25"/>
-    <mergeCell ref="A150:A153"/>
-    <mergeCell ref="E26:E29"/>
-    <mergeCell ref="D98:D101"/>
-    <mergeCell ref="C66:C69"/>
-    <mergeCell ref="A102:A105"/>
-    <mergeCell ref="E66:E69"/>
-    <mergeCell ref="D10:D13"/>
-    <mergeCell ref="B90:B93"/>
-    <mergeCell ref="D50:D53"/>
-    <mergeCell ref="F10:F13"/>
-    <mergeCell ref="A94:A97"/>
-    <mergeCell ref="B122:B125"/>
-    <mergeCell ref="F146:F149"/>
-    <mergeCell ref="E150:E153"/>
-    <mergeCell ref="D178:D181"/>
-    <mergeCell ref="D34:D37"/>
-    <mergeCell ref="F178:F181"/>
-    <mergeCell ref="C42:C45"/>
-    <mergeCell ref="F34:F37"/>
-    <mergeCell ref="A78:A81"/>
-    <mergeCell ref="F74:F77"/>
-    <mergeCell ref="E42:E45"/>
-    <mergeCell ref="B18:B21"/>
-    <mergeCell ref="B106:B109"/>
-    <mergeCell ref="F98:F101"/>
-    <mergeCell ref="C102:C105"/>
-    <mergeCell ref="A34:A37"/>
-    <mergeCell ref="B26:B29"/>
-    <mergeCell ref="F30:F33"/>
-    <mergeCell ref="A30:A33"/>
-    <mergeCell ref="B2:B5"/>
-    <mergeCell ref="D2:D5"/>
-    <mergeCell ref="B42:B45"/>
-    <mergeCell ref="C22:C25"/>
-    <mergeCell ref="E122:E125"/>
-    <mergeCell ref="F18:F21"/>
-    <mergeCell ref="B170:B173"/>
-    <mergeCell ref="E78:E81"/>
-    <mergeCell ref="A174:A177"/>
-    <mergeCell ref="D170:D173"/>
-    <mergeCell ref="B58:B61"/>
-    <mergeCell ref="F2:F5"/>
-    <mergeCell ref="E6:E9"/>
-    <mergeCell ref="C134:C137"/>
-    <mergeCell ref="F22:F25"/>
-    <mergeCell ref="C114:C117"/>
-    <mergeCell ref="A154:A157"/>
-    <mergeCell ref="E30:E33"/>
-    <mergeCell ref="E170:E173"/>
-    <mergeCell ref="E114:E117"/>
-    <mergeCell ref="F102:F105"/>
-    <mergeCell ref="C70:C73"/>
-    <mergeCell ref="E70:E73"/>
-    <mergeCell ref="C46:C49"/>
+    <mergeCell ref="F42:F45"/>
+    <mergeCell ref="D78:D81"/>
+    <mergeCell ref="E50:E53"/>
+    <mergeCell ref="D82:D85"/>
+    <mergeCell ref="C86:C89"/>
+    <mergeCell ref="F82:F85"/>
+    <mergeCell ref="C34:C37"/>
+    <mergeCell ref="D54:D57"/>
+    <mergeCell ref="C30:C33"/>
+    <mergeCell ref="E38:E41"/>
+    <mergeCell ref="D46:D49"/>
+    <mergeCell ref="C54:C57"/>
+    <mergeCell ref="F46:F49"/>
+    <mergeCell ref="E74:E77"/>
+    <mergeCell ref="A118:A121"/>
+    <mergeCell ref="C14:C17"/>
+    <mergeCell ref="B66:B69"/>
+    <mergeCell ref="C98:C101"/>
+    <mergeCell ref="C154:C157"/>
+    <mergeCell ref="E14:E17"/>
+    <mergeCell ref="A166:A169"/>
+    <mergeCell ref="E102:E105"/>
+    <mergeCell ref="B50:B53"/>
+    <mergeCell ref="A162:A165"/>
+    <mergeCell ref="A18:A21"/>
+    <mergeCell ref="D26:D29"/>
+    <mergeCell ref="A14:A17"/>
+    <mergeCell ref="C18:C21"/>
+    <mergeCell ref="B22:B25"/>
+    <mergeCell ref="D22:D25"/>
+    <mergeCell ref="E18:E21"/>
+    <mergeCell ref="B78:B81"/>
+    <mergeCell ref="A54:A57"/>
+    <mergeCell ref="A74:A77"/>
+    <mergeCell ref="B38:B41"/>
+    <mergeCell ref="A66:A69"/>
     <mergeCell ref="B30:B33"/>
     <mergeCell ref="C138:C141"/>
-    <mergeCell ref="C178:C181"/>
-    <mergeCell ref="E54:E57"/>
-    <mergeCell ref="D30:D33"/>
-    <mergeCell ref="E178:E181"/>
-    <mergeCell ref="D62:D65"/>
-    <mergeCell ref="D118:D121"/>
-    <mergeCell ref="F62:F65"/>
-    <mergeCell ref="E126:E129"/>
-    <mergeCell ref="C166:C169"/>
-    <mergeCell ref="C126:C129"/>
-    <mergeCell ref="C58:C61"/>
-    <mergeCell ref="E58:E61"/>
-    <mergeCell ref="D90:D93"/>
-    <mergeCell ref="B46:B49"/>
-    <mergeCell ref="B102:B105"/>
-    <mergeCell ref="E138:E141"/>
-    <mergeCell ref="D158:D161"/>
-    <mergeCell ref="B98:B101"/>
-    <mergeCell ref="F114:F117"/>
-    <mergeCell ref="D154:D157"/>
-    <mergeCell ref="C162:C165"/>
-    <mergeCell ref="B130:B133"/>
-    <mergeCell ref="B198:B201"/>
-    <mergeCell ref="D14:D17"/>
-    <mergeCell ref="A106:A109"/>
-    <mergeCell ref="F14:F17"/>
-    <mergeCell ref="B174:B177"/>
-    <mergeCell ref="A38:A41"/>
-    <mergeCell ref="B126:B129"/>
-    <mergeCell ref="D182:D185"/>
-    <mergeCell ref="D38:D41"/>
-    <mergeCell ref="F182:F185"/>
-    <mergeCell ref="A130:A133"/>
-    <mergeCell ref="A82:A85"/>
-    <mergeCell ref="B110:B113"/>
-    <mergeCell ref="E106:E109"/>
-    <mergeCell ref="D110:D113"/>
-    <mergeCell ref="B54:B57"/>
-    <mergeCell ref="E146:E149"/>
-    <mergeCell ref="A58:A61"/>
-    <mergeCell ref="F166:F169"/>
-    <mergeCell ref="E198:E201"/>
-    <mergeCell ref="C74:C77"/>
-    <mergeCell ref="A110:A113"/>
-    <mergeCell ref="F162:F165"/>
-    <mergeCell ref="B94:B97"/>
-    <mergeCell ref="F26:F29"/>
-    <mergeCell ref="C118:C121"/>
-    <mergeCell ref="F154:F157"/>
-    <mergeCell ref="A158:A161"/>
-    <mergeCell ref="D186:D189"/>
-    <mergeCell ref="A6:A9"/>
-    <mergeCell ref="A50:A53"/>
-    <mergeCell ref="C50:C53"/>
-    <mergeCell ref="B82:B85"/>
-    <mergeCell ref="A86:A89"/>
-    <mergeCell ref="F138:F141"/>
-    <mergeCell ref="C142:C145"/>
-    <mergeCell ref="F90:F93"/>
-    <mergeCell ref="E118:E121"/>
-    <mergeCell ref="B10:B13"/>
-    <mergeCell ref="E46:E49"/>
-    <mergeCell ref="D66:D69"/>
-    <mergeCell ref="D106:D109"/>
-    <mergeCell ref="B146:B149"/>
-    <mergeCell ref="F66:F69"/>
-    <mergeCell ref="D18:D21"/>
-    <mergeCell ref="D146:D149"/>
-    <mergeCell ref="E166:E169"/>
-    <mergeCell ref="A26:A29"/>
-    <mergeCell ref="F158:F161"/>
-    <mergeCell ref="B190:B193"/>
-    <mergeCell ref="D194:D197"/>
-    <mergeCell ref="B178:B181"/>
-    <mergeCell ref="E86:E89"/>
-    <mergeCell ref="B34:B37"/>
-    <mergeCell ref="F38:F41"/>
-    <mergeCell ref="A42:A45"/>
-    <mergeCell ref="B74:B77"/>
-    <mergeCell ref="F50:F53"/>
-    <mergeCell ref="E162:E165"/>
-    <mergeCell ref="D130:D133"/>
-    <mergeCell ref="A134:A137"/>
-    <mergeCell ref="B162:B165"/>
-    <mergeCell ref="F130:F133"/>
-    <mergeCell ref="D74:D77"/>
-    <mergeCell ref="E134:E137"/>
-    <mergeCell ref="D138:D141"/>
-    <mergeCell ref="F54:F57"/>
-    <mergeCell ref="C158:C161"/>
-    <mergeCell ref="F190:F193"/>
-    <mergeCell ref="E190:E193"/>
-    <mergeCell ref="B194:B197"/>
-    <mergeCell ref="A182:A185"/>
-    <mergeCell ref="F134:F137"/>
-    <mergeCell ref="E62:E65"/>
-    <mergeCell ref="E22:E25"/>
-    <mergeCell ref="C194:C197"/>
-    <mergeCell ref="C38:C41"/>
-    <mergeCell ref="D58:D61"/>
-    <mergeCell ref="A62:A65"/>
-    <mergeCell ref="F58:F61"/>
-    <mergeCell ref="A122:A125"/>
-    <mergeCell ref="C122:C125"/>
-    <mergeCell ref="C78:C81"/>
-    <mergeCell ref="D42:D45"/>
-    <mergeCell ref="A186:A189"/>
-    <mergeCell ref="C186:C189"/>
-    <mergeCell ref="D94:D97"/>
-    <mergeCell ref="E142:E145"/>
-    <mergeCell ref="E194:E197"/>
-    <mergeCell ref="B150:B153"/>
-    <mergeCell ref="A114:A117"/>
-    <mergeCell ref="A170:A173"/>
-    <mergeCell ref="A70:A73"/>
-    <mergeCell ref="C170:C173"/>
-    <mergeCell ref="F78:F81"/>
-    <mergeCell ref="F118:F121"/>
-    <mergeCell ref="C174:C177"/>
-    <mergeCell ref="F170:F173"/>
-    <mergeCell ref="B138:B141"/>
-    <mergeCell ref="D6:D9"/>
-    <mergeCell ref="C26:C29"/>
-    <mergeCell ref="D190:D193"/>
-    <mergeCell ref="B86:B89"/>
-    <mergeCell ref="A138:A141"/>
-    <mergeCell ref="E82:E85"/>
-    <mergeCell ref="D86:D89"/>
-    <mergeCell ref="F6:F9"/>
-    <mergeCell ref="F86:F89"/>
-    <mergeCell ref="F142:F145"/>
-    <mergeCell ref="C10:C13"/>
-    <mergeCell ref="B62:B65"/>
-    <mergeCell ref="E10:E13"/>
-    <mergeCell ref="B14:B17"/>
-    <mergeCell ref="B70:B73"/>
-    <mergeCell ref="D70:D73"/>
-    <mergeCell ref="E98:E101"/>
-    <mergeCell ref="F70:F73"/>
-    <mergeCell ref="E34:E37"/>
-    <mergeCell ref="B182:B185"/>
-    <mergeCell ref="D134:D137"/>
-    <mergeCell ref="C6:C9"/>
-    <mergeCell ref="C62:C65"/>
-    <mergeCell ref="A98:A101"/>
-    <mergeCell ref="F194:F197"/>
-    <mergeCell ref="A198:A201"/>
-    <mergeCell ref="C198:C201"/>
-    <mergeCell ref="D122:D125"/>
-    <mergeCell ref="C90:C93"/>
-    <mergeCell ref="A126:A129"/>
-    <mergeCell ref="D162:D165"/>
-    <mergeCell ref="C130:C133"/>
-    <mergeCell ref="F122:F125"/>
-    <mergeCell ref="C182:C185"/>
-    <mergeCell ref="A142:A145"/>
-    <mergeCell ref="E182:E185"/>
-    <mergeCell ref="C110:C113"/>
-    <mergeCell ref="F106:F109"/>
-    <mergeCell ref="A190:A193"/>
-    <mergeCell ref="C150:C153"/>
-    <mergeCell ref="F186:F189"/>
-    <mergeCell ref="C190:C193"/>
-    <mergeCell ref="B114:B117"/>
-    <mergeCell ref="D114:D117"/>
-    <mergeCell ref="B154:B157"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>